<commit_message>
Deploying to gh-pages from @ dieghernan/dieghernan.github.io@c2953f32f1ea383c3f5cd6eb1c663097fa308779 🚀
</commit_message>
<xml_diff>
--- a/assets/data/flights.xlsx
+++ b/assets/data/flights.xlsx
@@ -1,30 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C352842-DA4D-4AEA-ADF1-C558DEC4C834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="51">
   <si>
     <t>start</t>
   </si>
@@ -174,12 +170,15 @@
   </si>
   <si>
     <t>Rome</t>
+  </si>
+  <si>
+    <t>Bristol</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -490,17 +489,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F188"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F204"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -520,7 +519,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -540,7 +539,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -560,7 +559,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -580,7 +579,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
@@ -600,7 +599,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
@@ -620,7 +619,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>3</v>
       </c>
@@ -640,7 +639,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>4</v>
       </c>
@@ -660,7 +659,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>4</v>
       </c>
@@ -680,7 +679,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>5</v>
       </c>
@@ -700,7 +699,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>5</v>
       </c>
@@ -720,7 +719,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>6</v>
       </c>
@@ -740,7 +739,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>6</v>
       </c>
@@ -760,7 +759,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>6</v>
       </c>
@@ -780,7 +779,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>7</v>
       </c>
@@ -800,7 +799,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>8</v>
       </c>
@@ -820,7 +819,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>8</v>
       </c>
@@ -840,7 +839,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>9</v>
       </c>
@@ -860,7 +859,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>9</v>
       </c>
@@ -880,7 +879,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>10</v>
       </c>
@@ -900,7 +899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>10</v>
       </c>
@@ -920,7 +919,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>11</v>
       </c>
@@ -940,7 +939,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>12</v>
       </c>
@@ -960,7 +959,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>12</v>
       </c>
@@ -980,7 +979,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>13</v>
       </c>
@@ -1000,7 +999,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>13</v>
       </c>
@@ -1020,7 +1019,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>14</v>
       </c>
@@ -1040,7 +1039,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>14</v>
       </c>
@@ -1060,7 +1059,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <f t="shared" ref="A29:A93" si="0">A27+1</f>
         <v>15</v>
@@ -1081,7 +1080,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1102,7 +1101,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1123,7 +1122,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1144,7 +1143,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1165,7 +1164,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1186,7 +1185,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1207,7 +1206,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1228,7 +1227,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1249,7 +1248,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <f>A37+1</f>
         <v>20</v>
@@ -1270,7 +1269,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <f>A38</f>
         <v>20</v>
@@ -1291,7 +1290,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1312,7 +1311,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1333,7 +1332,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -1354,7 +1353,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -1375,7 +1374,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -1396,7 +1395,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -1417,7 +1416,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -1438,7 +1437,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -1459,7 +1458,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -1480,7 +1479,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -1501,7 +1500,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -1522,7 +1521,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -1543,7 +1542,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -1564,7 +1563,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -1585,7 +1584,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -1606,7 +1605,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -1627,7 +1626,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -1648,7 +1647,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -1669,7 +1668,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -1690,7 +1689,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -1711,7 +1710,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -1732,7 +1731,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -1753,7 +1752,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -1774,7 +1773,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -1795,7 +1794,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -1816,7 +1815,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -1837,7 +1836,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -1858,7 +1857,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -1879,7 +1878,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -1900,7 +1899,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -1921,7 +1920,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -1942,7 +1941,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -1963,7 +1962,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -1984,7 +1983,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -2005,7 +2004,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -2026,7 +2025,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -2047,7 +2046,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -2068,7 +2067,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -2089,7 +2088,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -2110,7 +2109,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -2131,7 +2130,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -2152,7 +2151,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -2173,7 +2172,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -2194,7 +2193,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -2215,7 +2214,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -2236,7 +2235,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -2257,7 +2256,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -2278,7 +2277,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -2299,7 +2298,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -2320,7 +2319,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -2341,7 +2340,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -2362,7 +2361,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -2383,7 +2382,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -2404,7 +2403,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -2425,7 +2424,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <f t="shared" ref="A94:A117" si="1">A92+1</f>
         <v>48</v>
@@ -2446,7 +2445,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95">
         <f t="shared" si="1"/>
         <v>48</v>
@@ -2467,7 +2466,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96">
         <f t="shared" si="1"/>
         <v>49</v>
@@ -2488,7 +2487,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97">
         <f t="shared" si="1"/>
         <v>49</v>
@@ -2509,7 +2508,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98">
         <f t="shared" si="1"/>
         <v>50</v>
@@ -2530,7 +2529,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99">
         <f t="shared" si="1"/>
         <v>50</v>
@@ -2551,7 +2550,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100">
         <f t="shared" si="1"/>
         <v>51</v>
@@ -2572,7 +2571,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101">
         <f t="shared" si="1"/>
         <v>51</v>
@@ -2593,7 +2592,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102">
         <f t="shared" si="1"/>
         <v>52</v>
@@ -2614,7 +2613,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103">
         <f t="shared" si="1"/>
         <v>52</v>
@@ -2635,7 +2634,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104">
         <f t="shared" si="1"/>
         <v>53</v>
@@ -2656,7 +2655,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105">
         <f t="shared" si="1"/>
         <v>53</v>
@@ -2677,7 +2676,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106">
         <f t="shared" si="1"/>
         <v>54</v>
@@ -2698,7 +2697,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107">
         <f t="shared" si="1"/>
         <v>54</v>
@@ -2719,7 +2718,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108">
         <f t="shared" si="1"/>
         <v>55</v>
@@ -2740,7 +2739,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109">
         <f t="shared" si="1"/>
         <v>55</v>
@@ -2761,7 +2760,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110">
         <f t="shared" si="1"/>
         <v>56</v>
@@ -2782,7 +2781,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111">
         <f t="shared" si="1"/>
         <v>56</v>
@@ -2803,7 +2802,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112">
         <f t="shared" si="1"/>
         <v>57</v>
@@ -2824,7 +2823,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113">
         <f t="shared" si="1"/>
         <v>57</v>
@@ -2845,7 +2844,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114">
         <f t="shared" si="1"/>
         <v>58</v>
@@ -2866,7 +2865,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115">
         <f t="shared" si="1"/>
         <v>58</v>
@@ -2887,7 +2886,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116">
         <f t="shared" si="1"/>
         <v>59</v>
@@ -2908,7 +2907,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117">
         <f t="shared" si="1"/>
         <v>59</v>
@@ -2929,7 +2928,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118">
         <f t="shared" ref="A118:A119" si="2">A116+1</f>
         <v>60</v>
@@ -2950,7 +2949,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119">
         <f t="shared" si="2"/>
         <v>60</v>
@@ -2971,7 +2970,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120">
         <f t="shared" ref="A120:A178" si="3">A118+1</f>
         <v>61</v>
@@ -2992,7 +2991,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121">
         <f t="shared" si="3"/>
         <v>61</v>
@@ -3013,7 +3012,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122">
         <f t="shared" si="3"/>
         <v>62</v>
@@ -3034,7 +3033,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123">
         <f t="shared" si="3"/>
         <v>62</v>
@@ -3055,7 +3054,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124">
         <f t="shared" si="3"/>
         <v>63</v>
@@ -3076,7 +3075,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125">
         <f t="shared" si="3"/>
         <v>63</v>
@@ -3097,7 +3096,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126">
         <f>A125</f>
         <v>63</v>
@@ -3118,7 +3117,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127">
         <f>A126</f>
         <v>63</v>
@@ -3139,7 +3138,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128">
         <f t="shared" ref="A128:A134" si="4">A127</f>
         <v>63</v>
@@ -3160,7 +3159,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129">
         <f t="shared" si="4"/>
         <v>63</v>
@@ -3181,7 +3180,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130">
         <f t="shared" si="4"/>
         <v>63</v>
@@ -3202,7 +3201,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131">
         <f t="shared" si="4"/>
         <v>63</v>
@@ -3223,7 +3222,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132">
         <f>A131</f>
         <v>63</v>
@@ -3244,7 +3243,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133">
         <f>A132+1</f>
         <v>64</v>
@@ -3265,7 +3264,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134">
         <f t="shared" si="4"/>
         <v>64</v>
@@ -3286,7 +3285,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135">
         <f t="shared" si="3"/>
         <v>65</v>
@@ -3307,7 +3306,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136">
         <f t="shared" si="3"/>
         <v>65</v>
@@ -3328,7 +3327,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137">
         <f t="shared" si="3"/>
         <v>66</v>
@@ -3349,7 +3348,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138">
         <f t="shared" si="3"/>
         <v>66</v>
@@ -3370,7 +3369,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139">
         <f t="shared" si="3"/>
         <v>67</v>
@@ -3391,7 +3390,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140">
         <f t="shared" si="3"/>
         <v>67</v>
@@ -3412,7 +3411,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141">
         <f t="shared" si="3"/>
         <v>68</v>
@@ -3433,7 +3432,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142">
         <f t="shared" si="3"/>
         <v>68</v>
@@ -3454,7 +3453,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143">
         <f>A142</f>
         <v>68</v>
@@ -3475,7 +3474,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144">
         <f t="shared" si="3"/>
         <v>69</v>
@@ -3496,7 +3495,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145">
         <f t="shared" si="3"/>
         <v>69</v>
@@ -3517,7 +3516,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146">
         <f t="shared" si="3"/>
         <v>70</v>
@@ -3538,7 +3537,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147">
         <f t="shared" si="3"/>
         <v>70</v>
@@ -3559,7 +3558,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148">
         <f t="shared" si="3"/>
         <v>71</v>
@@ -3580,7 +3579,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149">
         <f t="shared" si="3"/>
         <v>71</v>
@@ -3601,7 +3600,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150">
         <f>A149</f>
         <v>71</v>
@@ -3622,7 +3621,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151">
         <f>A150</f>
         <v>71</v>
@@ -3643,7 +3642,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152">
         <f t="shared" si="3"/>
         <v>72</v>
@@ -3664,7 +3663,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153">
         <f t="shared" si="3"/>
         <v>72</v>
@@ -3685,7 +3684,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154">
         <f>A153</f>
         <v>72</v>
@@ -3706,7 +3705,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155">
         <f t="shared" si="3"/>
         <v>73</v>
@@ -3727,7 +3726,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156">
         <f t="shared" si="3"/>
         <v>73</v>
@@ -3748,7 +3747,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157">
         <f>A156</f>
         <v>73</v>
@@ -3769,7 +3768,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158">
         <f t="shared" si="3"/>
         <v>74</v>
@@ -3790,7 +3789,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159">
         <f t="shared" si="3"/>
         <v>74</v>
@@ -3811,7 +3810,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160">
         <f t="shared" si="3"/>
         <v>75</v>
@@ -3832,7 +3831,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161">
         <f t="shared" si="3"/>
         <v>75</v>
@@ -3853,7 +3852,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162">
         <f t="shared" si="3"/>
         <v>76</v>
@@ -3874,7 +3873,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163">
         <f t="shared" si="3"/>
         <v>76</v>
@@ -3895,7 +3894,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164">
         <f t="shared" si="3"/>
         <v>77</v>
@@ -3916,7 +3915,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165">
         <f t="shared" si="3"/>
         <v>77</v>
@@ -3937,7 +3936,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166">
         <f t="shared" si="3"/>
         <v>78</v>
@@ -3958,7 +3957,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167">
         <f t="shared" si="3"/>
         <v>78</v>
@@ -3979,7 +3978,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168">
         <f t="shared" si="3"/>
         <v>79</v>
@@ -4000,7 +3999,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169">
         <f>A168+1</f>
         <v>80</v>
@@ -4021,7 +4020,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170">
         <f t="shared" si="3"/>
         <v>80</v>
@@ -4042,7 +4041,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171">
         <f t="shared" si="3"/>
         <v>81</v>
@@ -4063,7 +4062,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172">
         <f t="shared" si="3"/>
         <v>81</v>
@@ -4084,7 +4083,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173">
         <f t="shared" si="3"/>
         <v>82</v>
@@ -4105,7 +4104,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174">
         <f t="shared" si="3"/>
         <v>82</v>
@@ -4126,7 +4125,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175">
         <f t="shared" si="3"/>
         <v>83</v>
@@ -4147,7 +4146,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176">
         <f t="shared" si="3"/>
         <v>83</v>
@@ -4168,7 +4167,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177">
         <f t="shared" si="3"/>
         <v>84</v>
@@ -4189,7 +4188,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178">
         <f t="shared" si="3"/>
         <v>84</v>
@@ -4210,7 +4209,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179">
         <f t="shared" ref="A179:A186" si="5">A177+1</f>
         <v>85</v>
@@ -4231,7 +4230,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180">
         <f t="shared" si="5"/>
         <v>85</v>
@@ -4252,7 +4251,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181">
         <f t="shared" si="5"/>
         <v>86</v>
@@ -4273,7 +4272,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182">
         <f t="shared" si="5"/>
         <v>86</v>
@@ -4294,7 +4293,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183">
         <f t="shared" si="5"/>
         <v>87</v>
@@ -4315,7 +4314,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184">
         <f t="shared" si="5"/>
         <v>87</v>
@@ -4336,7 +4335,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185">
         <f t="shared" si="5"/>
         <v>88</v>
@@ -4357,7 +4356,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186">
         <f t="shared" si="5"/>
         <v>88</v>
@@ -4378,7 +4377,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>89</v>
       </c>
@@ -4398,7 +4397,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>89</v>
       </c>
@@ -4416,6 +4415,326 @@
       </c>
       <c r="F188" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A189">
+        <v>90</v>
+      </c>
+      <c r="B189" t="s">
+        <v>4</v>
+      </c>
+      <c r="C189" t="s">
+        <v>44</v>
+      </c>
+      <c r="D189">
+        <v>6</v>
+      </c>
+      <c r="E189">
+        <v>2022</v>
+      </c>
+      <c r="F189" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A190">
+        <v>90</v>
+      </c>
+      <c r="B190" t="s">
+        <v>44</v>
+      </c>
+      <c r="C190" t="s">
+        <v>4</v>
+      </c>
+      <c r="D190">
+        <v>6</v>
+      </c>
+      <c r="E190">
+        <v>2022</v>
+      </c>
+      <c r="F190" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A191">
+        <v>91</v>
+      </c>
+      <c r="B191" t="s">
+        <v>4</v>
+      </c>
+      <c r="C191" t="s">
+        <v>50</v>
+      </c>
+      <c r="D191">
+        <v>8</v>
+      </c>
+      <c r="E191">
+        <v>2022</v>
+      </c>
+      <c r="F191" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A192">
+        <v>91</v>
+      </c>
+      <c r="B192" t="s">
+        <v>50</v>
+      </c>
+      <c r="C192" t="s">
+        <v>4</v>
+      </c>
+      <c r="D192">
+        <v>8</v>
+      </c>
+      <c r="E192">
+        <v>2022</v>
+      </c>
+      <c r="F192" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A193">
+        <v>92</v>
+      </c>
+      <c r="B193" t="s">
+        <v>4</v>
+      </c>
+      <c r="C193" t="s">
+        <v>44</v>
+      </c>
+      <c r="D193">
+        <v>10</v>
+      </c>
+      <c r="E193">
+        <v>2022</v>
+      </c>
+      <c r="F193" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A194">
+        <v>92</v>
+      </c>
+      <c r="B194" t="s">
+        <v>44</v>
+      </c>
+      <c r="C194" t="s">
+        <v>4</v>
+      </c>
+      <c r="D194">
+        <v>10</v>
+      </c>
+      <c r="E194">
+        <v>2022</v>
+      </c>
+      <c r="F194" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A195">
+        <v>93</v>
+      </c>
+      <c r="B195" t="s">
+        <v>4</v>
+      </c>
+      <c r="C195" t="s">
+        <v>5</v>
+      </c>
+      <c r="D195">
+        <v>6</v>
+      </c>
+      <c r="E195">
+        <v>2023</v>
+      </c>
+      <c r="F195" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A196">
+        <v>93</v>
+      </c>
+      <c r="B196" t="s">
+        <v>5</v>
+      </c>
+      <c r="C196" t="s">
+        <v>4</v>
+      </c>
+      <c r="D196">
+        <v>6</v>
+      </c>
+      <c r="E196">
+        <v>2023</v>
+      </c>
+      <c r="F196" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A197">
+        <v>94</v>
+      </c>
+      <c r="B197" t="s">
+        <v>4</v>
+      </c>
+      <c r="C197" t="s">
+        <v>5</v>
+      </c>
+      <c r="D197">
+        <v>9</v>
+      </c>
+      <c r="E197">
+        <v>2023</v>
+      </c>
+      <c r="F197" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A198">
+        <v>94</v>
+      </c>
+      <c r="B198" t="s">
+        <v>5</v>
+      </c>
+      <c r="C198" t="s">
+        <v>4</v>
+      </c>
+      <c r="D198">
+        <v>9</v>
+      </c>
+      <c r="E198">
+        <v>2023</v>
+      </c>
+      <c r="F198" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A199">
+        <v>95</v>
+      </c>
+      <c r="B199" t="s">
+        <v>4</v>
+      </c>
+      <c r="C199" t="s">
+        <v>44</v>
+      </c>
+      <c r="D199">
+        <v>12</v>
+      </c>
+      <c r="E199">
+        <v>2023</v>
+      </c>
+      <c r="F199" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A200">
+        <v>95</v>
+      </c>
+      <c r="B200" t="s">
+        <v>44</v>
+      </c>
+      <c r="C200" t="s">
+        <v>4</v>
+      </c>
+      <c r="D200">
+        <v>12</v>
+      </c>
+      <c r="E200">
+        <v>2023</v>
+      </c>
+      <c r="F200" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A201">
+        <v>96</v>
+      </c>
+      <c r="B201" t="s">
+        <v>4</v>
+      </c>
+      <c r="C201" t="s">
+        <v>22</v>
+      </c>
+      <c r="D201">
+        <v>3</v>
+      </c>
+      <c r="E201">
+        <v>2024</v>
+      </c>
+      <c r="F201" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A202">
+        <v>96</v>
+      </c>
+      <c r="B202" t="s">
+        <v>22</v>
+      </c>
+      <c r="C202" t="s">
+        <v>4</v>
+      </c>
+      <c r="D202">
+        <v>3</v>
+      </c>
+      <c r="E202">
+        <v>2024</v>
+      </c>
+      <c r="F202" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A203">
+        <v>97</v>
+      </c>
+      <c r="B203" t="s">
+        <v>4</v>
+      </c>
+      <c r="C203" t="s">
+        <v>26</v>
+      </c>
+      <c r="D203">
+        <v>5</v>
+      </c>
+      <c r="E203">
+        <v>2024</v>
+      </c>
+      <c r="F203" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A204">
+        <v>97</v>
+      </c>
+      <c r="B204" t="s">
+        <v>26</v>
+      </c>
+      <c r="C204" t="s">
+        <v>4</v>
+      </c>
+      <c r="D204">
+        <v>5</v>
+      </c>
+      <c r="E204">
+        <v>2024</v>
+      </c>
+      <c r="F204" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>